<commit_message>
Change german wording to english
</commit_message>
<xml_diff>
--- a/data/raw_erp_export.xlsx
+++ b/data/raw_erp_export.xlsx
@@ -488,7 +488,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Verkauf Fertigarzneimittel an Vertriebsgesellschaft US05</t>
+          <t>Sale of finished pharmaceuticals to distributor US05</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -533,7 +533,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Verkauf Fertigarzneimittel an Vertriebsgesellschaft US05</t>
+          <t>Sale of finished pharmaceuticals to distributor US05</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -578,7 +578,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Verkauf Fertigarzneimittel an Vertriebsgesellschaft US05</t>
+          <t>Sale of finished pharmaceuticals to distributor US05</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -623,7 +623,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Verkauf Fertigarzneimittel an Vertriebsgesellschaft US05</t>
+          <t>Sale of finished pharmaceuticals to distributor US05</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -668,7 +668,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Verkauf Fertigarzneimittel an Vertriebsgesellschaft US05</t>
+          <t>Sale of finished pharmaceuticals to distributor US05</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -713,7 +713,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Verkauf Fertigarzneimittel an Vertriebsgesellschaft US05</t>
+          <t>Sale of finished pharmaceuticals to distributor US05</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -758,7 +758,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Verkauf Fertigarzneimittel an Vertriebsgesellschaft US05</t>
+          <t>Sale of finished pharmaceuticals to distributor US05</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -803,7 +803,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Verkauf Fertigarzneimittel an Vertriebsgesellschaft US05</t>
+          <t>Sale of finished pharmaceuticals to distributor US05</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -848,7 +848,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Verkauf Fertigarzneimittel an Vertriebsgesellschaft US05</t>
+          <t>Sale of finished pharmaceuticals to distributor US05</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -893,7 +893,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Verkauf Fertigarzneimittel an Vertriebsgesellschaft US05</t>
+          <t>Sale of finished pharmaceuticals to distributor US05</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -938,7 +938,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Verkauf Fertigarzneimittel an Vertriebsgesellschaft US05</t>
+          <t>Sale of finished pharmaceuticals to distributor US05</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -983,7 +983,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Verkauf Fertigarzneimittel an Vertriebsgesellschaft US05</t>
+          <t>Sale of finished pharmaceuticals to distributor US05</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -1028,7 +1028,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Verkauf Fertigarzneimittel an Vertriebsgesellschaft US05</t>
+          <t>Sale of finished pharmaceuticals to distributor US05</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -1073,7 +1073,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Verkauf Fertigarzneimittel an Vertriebsgesellschaft US05</t>
+          <t>Sale of finished pharmaceuticals to distributor US05</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -1118,7 +1118,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Verkauf Fertigarzneimittel an Vertriebsgesellschaft US05</t>
+          <t>Sale of finished pharmaceuticals to distributor US05</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -1163,7 +1163,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Verkauf Fertigarzneimittel an Vertriebsgesellschaft US05</t>
+          <t>Sale of finished pharmaceuticals to distributor US05</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -1208,7 +1208,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Verkauf Fertigware an Grosshaendler McKesson Specialty Distribution</t>
+          <t>Sale of finished goods to wholesaler McKesson Specialty Distribution</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -1249,7 +1249,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Verkauf Fertigware an Grosshaendler Cardinal Health East</t>
+          <t>Sale of finished goods to wholesaler Cardinal Health East</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -1290,7 +1290,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Verkauf Fertigware an Grosshaendler AmerisourceBergen Pharma</t>
+          <t>Sale of finished goods to wholesaler AmerisourceBergen Pharma</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -1331,7 +1331,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Verkauf Fertigware an Grosshaendler McKesson Specialty Distribution</t>
+          <t>Sale of finished goods to wholesaler McKesson Specialty Distribution</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -1372,7 +1372,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Verkauf Fertigware an Grosshaendler AmerisourceBergen Pharma</t>
+          <t>Sale of finished goods to wholesaler AmerisourceBergen Pharma</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -1413,7 +1413,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Verkauf Fertigware an Grosshaendler AmerisourceBergen Pharma</t>
+          <t>Sale of finished goods to wholesaler AmerisourceBergen Pharma</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -1454,7 +1454,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Verkauf Fertigware an Grosshaendler AmerisourceBergen Pharma</t>
+          <t>Sale of finished goods to wholesaler AmerisourceBergen Pharma</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -1495,7 +1495,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Verkauf Fertigware an Grosshaendler McKesson Specialty Distribution</t>
+          <t>Sale of finished goods to wholesaler McKesson Specialty Distribution</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -1536,7 +1536,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Verkauf Fertigware an Grosshaendler AmerisourceBergen Pharma</t>
+          <t>Sale of finished goods to wholesaler AmerisourceBergen Pharma</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -1577,7 +1577,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Verkauf Fertigware an Grosshaendler AmerisourceBergen Pharma</t>
+          <t>Sale of finished goods to wholesaler AmerisourceBergen Pharma</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -1618,7 +1618,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Verkauf Fertigware an Grosshaendler McKesson Specialty Distribution</t>
+          <t>Sale of finished goods to wholesaler McKesson Specialty Distribution</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -1659,7 +1659,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Verkauf Fertigware an Grosshaendler AmerisourceBergen Pharma</t>
+          <t>Sale of finished goods to wholesaler AmerisourceBergen Pharma</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -1700,7 +1700,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Verkauf Fertigware an Grosshaendler Cardinal Health East</t>
+          <t>Sale of finished goods to wholesaler Cardinal Health East</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -1741,7 +1741,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Verkauf Fertigware an Grosshaendler McKesson Specialty Distribution</t>
+          <t>Sale of finished goods to wholesaler McKesson Specialty Distribution</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -1782,7 +1782,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Verkauf Fertigware an Grosshaendler McKesson Specialty Distribution</t>
+          <t>Sale of finished goods to wholesaler McKesson Specialty Distribution</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -1823,7 +1823,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Verkauf Fertigware an Grosshaendler AmerisourceBergen Pharma</t>
+          <t>Sale of finished goods to wholesaler AmerisourceBergen Pharma</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -1864,7 +1864,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Verkauf Fertigware an Grosshaendler McKesson Specialty Distribution</t>
+          <t>Sale of finished goods to wholesaler McKesson Specialty Distribution</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -1905,7 +1905,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Verkauf Fertigware an Grosshaendler AmerisourceBergen Pharma</t>
+          <t>Sale of finished goods to wholesaler AmerisourceBergen Pharma</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -1946,7 +1946,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Verkauf Fertigware an Grosshaendler AmerisourceBergen Pharma</t>
+          <t>Sale of finished goods to wholesaler AmerisourceBergen Pharma</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -1987,7 +1987,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Verkauf Fertigware an Grosshaendler McKesson Specialty Distribution</t>
+          <t>Sale of finished goods to wholesaler McKesson Specialty Distribution</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -2028,7 +2028,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Gutschrift Retoure Grosshandel</t>
+          <t>Credit note wholesale return</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -2069,7 +2069,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Verkauf Fertigarzneimittel an Vertriebsgesellschaft DE01</t>
+          <t>Sale of finished pharmaceuticals to distributor DE01</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -2114,7 +2114,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Verkauf Fertigarzneimittel an Vertriebsgesellschaft DE01</t>
+          <t>Sale of finished pharmaceuticals to distributor DE01</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -2159,7 +2159,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Verkauf Fertigarzneimittel an Vertriebsgesellschaft DE01</t>
+          <t>Sale of finished pharmaceuticals to distributor DE01</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -2204,7 +2204,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Verkauf Fertigarzneimittel an Vertriebsgesellschaft DE01</t>
+          <t>Sale of finished pharmaceuticals to distributor DE01</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -2249,7 +2249,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Verkauf Fertigarzneimittel an Vertriebsgesellschaft DE01</t>
+          <t>Sale of finished pharmaceuticals to distributor DE01</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -2294,7 +2294,7 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Verkauf Fertigarzneimittel an Vertriebsgesellschaft DE01</t>
+          <t>Sale of finished pharmaceuticals to distributor DE01</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -2339,7 +2339,7 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Verkauf Fertigarzneimittel an Vertriebsgesellschaft DE01</t>
+          <t>Sale of finished pharmaceuticals to distributor DE01</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -2384,7 +2384,7 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Verkauf Fertigarzneimittel an Vertriebsgesellschaft DE01</t>
+          <t>Sale of finished pharmaceuticals to distributor DE01</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
@@ -2429,7 +2429,7 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Verkauf Fertigarzneimittel an Vertriebsgesellschaft DE01</t>
+          <t>Sale of finished pharmaceuticals to distributor DE01</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -2474,7 +2474,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Verkauf Fertigarzneimittel an Vertriebsgesellschaft DE01</t>
+          <t>Sale of finished pharmaceuticals to distributor DE01</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -2519,7 +2519,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Verkauf Fertigarzneimittel an Vertriebsgesellschaft DE01</t>
+          <t>Sale of finished pharmaceuticals to distributor DE01</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -2564,7 +2564,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Verkauf Fertigarzneimittel an Vertriebsgesellschaft DE01</t>
+          <t>Sale of finished pharmaceuticals to distributor DE01</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
@@ -2609,7 +2609,7 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Verkauf Fertigarzneimittel an Vertriebsgesellschaft DE01</t>
+          <t>Sale of finished pharmaceuticals to distributor DE01</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -2654,7 +2654,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Verkauf Fertigarzneimittel an Vertriebsgesellschaft DE01</t>
+          <t>Sale of finished pharmaceuticals to distributor DE01</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
@@ -2699,7 +2699,7 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Verkauf Fertigarzneimittel an Vertriebsgesellschaft DE01</t>
+          <t>Sale of finished pharmaceuticals to distributor DE01</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
@@ -2744,7 +2744,7 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Verkauf Fertigarzneimittel an Vertriebsgesellschaft DE01</t>
+          <t>Sale of finished pharmaceuticals to distributor DE01</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -2789,7 +2789,7 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Verkauf Fertigarzneimittel an Vertriebsgesellschaft DE01</t>
+          <t>Sale of finished pharmaceuticals to distributor DE01</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
@@ -2834,7 +2834,7 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Verkauf Fertigarzneimittel an Vertriebsgesellschaft DE01</t>
+          <t>Sale of finished pharmaceuticals to distributor DE01</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
@@ -2879,7 +2879,7 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Verkauf Fertigarzneimittel an Vertriebsgesellschaft DE01</t>
+          <t>Sale of finished pharmaceuticals to distributor DE01</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
@@ -2924,7 +2924,7 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Verkauf Fertigarzneimittel an Vertriebsgesellschaft DE01</t>
+          <t>Sale of finished pharmaceuticals to distributor DE01</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
@@ -2969,7 +2969,7 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Verkauf Fertigware an Grosshaendler Apothekengenossenschaft Nord</t>
+          <t>Sale of finished goods to wholesaler Apothekengenossenschaft Nord</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
@@ -3010,7 +3010,7 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Verkauf Fertigware an Grosshaendler MedGross Deutschland</t>
+          <t>Sale of finished goods to wholesaler MedGross Deutschland</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
@@ -3051,7 +3051,7 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Verkauf Fertigware an Grosshaendler Phoenix Pharmahandel AG</t>
+          <t>Sale of finished goods to wholesaler Phoenix Pharmahandel AG</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
@@ -3092,7 +3092,7 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Verkauf Fertigware an Grosshaendler MedGross Deutschland</t>
+          <t>Sale of finished goods to wholesaler MedGross Deutschland</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
@@ -3133,7 +3133,7 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Verkauf Fertigware an Grosshaendler Phoenix Pharmahandel AG</t>
+          <t>Sale of finished goods to wholesaler Phoenix Pharmahandel AG</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
@@ -3174,7 +3174,7 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Verkauf Fertigware an Grosshaendler Phoenix Pharmahandel AG</t>
+          <t>Sale of finished goods to wholesaler Phoenix Pharmahandel AG</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
@@ -3215,7 +3215,7 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Verkauf Fertigware an Grosshaendler Apothekengenossenschaft Nord</t>
+          <t>Sale of finished goods to wholesaler Apothekengenossenschaft Nord</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
@@ -3256,7 +3256,7 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Verkauf Fertigware an Grosshaendler Phoenix Pharmahandel AG</t>
+          <t>Sale of finished goods to wholesaler Phoenix Pharmahandel AG</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
@@ -3297,7 +3297,7 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Verkauf Fertigware an Grosshaendler Apothekengenossenschaft Nord</t>
+          <t>Sale of finished goods to wholesaler Apothekengenossenschaft Nord</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
@@ -3338,7 +3338,7 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Verkauf Fertigware an Grosshaendler Apothekengenossenschaft Nord</t>
+          <t>Sale of finished goods to wholesaler Apothekengenossenschaft Nord</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
@@ -3379,7 +3379,7 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Verkauf Fertigware an Grosshaendler MedGross Deutschland</t>
+          <t>Sale of finished goods to wholesaler MedGross Deutschland</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
@@ -3420,7 +3420,7 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Verkauf Fertigware an Grosshaendler Phoenix Pharmahandel AG</t>
+          <t>Sale of finished goods to wholesaler Phoenix Pharmahandel AG</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
@@ -3461,7 +3461,7 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Verkauf Fertigware an Grosshaendler Apothekengenossenschaft Nord</t>
+          <t>Sale of finished goods to wholesaler Apothekengenossenschaft Nord</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
@@ -3502,7 +3502,7 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Verkauf Fertigware an Grosshaendler MedGross Deutschland</t>
+          <t>Sale of finished goods to wholesaler MedGross Deutschland</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
@@ -3543,7 +3543,7 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Verkauf Fertigware an Grosshaendler Phoenix Pharmahandel AG</t>
+          <t>Sale of finished goods to wholesaler Phoenix Pharmahandel AG</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
@@ -3584,7 +3584,7 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>Verkauf Fertigware an Grosshaendler Phoenix Pharmahandel AG</t>
+          <t>Sale of finished goods to wholesaler Phoenix Pharmahandel AG</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
@@ -3625,7 +3625,7 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Verkauf Fertigware an Grosshaendler MedGross Deutschland</t>
+          <t>Sale of finished goods to wholesaler MedGross Deutschland</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
@@ -3666,7 +3666,7 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Verkauf Fertigware an Grosshaendler MedGross Deutschland</t>
+          <t>Sale of finished goods to wholesaler MedGross Deutschland</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
@@ -3707,7 +3707,7 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Verkauf Fertigware an Grosshaendler Apothekengenossenschaft Nord</t>
+          <t>Sale of finished goods to wholesaler Apothekengenossenschaft Nord</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
@@ -3748,7 +3748,7 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>Verkauf Fertigware an Grosshaendler MedGross Deutschland</t>
+          <t>Sale of finished goods to wholesaler MedGross Deutschland</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
@@ -3789,7 +3789,7 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Verkauf Fertigware an Grosshaendler MedGross Deutschland</t>
+          <t>Sale of finished goods to wholesaler MedGross Deutschland</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
@@ -3830,7 +3830,7 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Verkauf Fertigware an Grosshaendler Phoenix Pharmahandel AG</t>
+          <t>Sale of finished goods to wholesaler Phoenix Pharmahandel AG</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
@@ -3871,7 +3871,7 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Verkauf Fertigware an Grosshaendler MedGross Deutschland</t>
+          <t>Sale of finished goods to wholesaler MedGross Deutschland</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
@@ -3912,7 +3912,7 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Gutschrift Retoure Grosshandel</t>
+          <t>Credit note wholesale return</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
@@ -3953,7 +3953,7 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Verkauf Fertigarzneimittel an Vertriebsgesellschaft FR03</t>
+          <t>Sale of finished pharmaceuticals to distributor FR03</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
@@ -3998,7 +3998,7 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Verkauf Fertigarzneimittel an Vertriebsgesellschaft FR03</t>
+          <t>Sale of finished pharmaceuticals to distributor FR03</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
@@ -4043,7 +4043,7 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>Verkauf Fertigarzneimittel an Vertriebsgesellschaft FR03</t>
+          <t>Sale of finished pharmaceuticals to distributor FR03</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
@@ -4088,7 +4088,7 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Verkauf Fertigarzneimittel an Vertriebsgesellschaft FR03</t>
+          <t>Sale of finished pharmaceuticals to distributor FR03</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
@@ -4133,7 +4133,7 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>Verkauf Fertigarzneimittel an Vertriebsgesellschaft FR03</t>
+          <t>Sale of finished pharmaceuticals to distributor FR03</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
@@ -4178,7 +4178,7 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>Verkauf Fertigarzneimittel an Vertriebsgesellschaft FR03</t>
+          <t>Sale of finished pharmaceuticals to distributor FR03</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
@@ -4223,7 +4223,7 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>Verkauf Fertigarzneimittel an Vertriebsgesellschaft FR03</t>
+          <t>Sale of finished pharmaceuticals to distributor FR03</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
@@ -4268,7 +4268,7 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>Verkauf Fertigarzneimittel an Vertriebsgesellschaft FR03</t>
+          <t>Sale of finished pharmaceuticals to distributor FR03</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
@@ -4313,7 +4313,7 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>Verkauf Fertigarzneimittel an Vertriebsgesellschaft FR03</t>
+          <t>Sale of finished pharmaceuticals to distributor FR03</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
@@ -4358,7 +4358,7 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>Verkauf Fertigarzneimittel an Vertriebsgesellschaft FR03</t>
+          <t>Sale of finished pharmaceuticals to distributor FR03</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
@@ -4403,7 +4403,7 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>Verkauf Fertigarzneimittel an Vertriebsgesellschaft FR03</t>
+          <t>Sale of finished pharmaceuticals to distributor FR03</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
@@ -4448,7 +4448,7 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>Verkauf Fertigarzneimittel an Vertriebsgesellschaft FR03</t>
+          <t>Sale of finished pharmaceuticals to distributor FR03</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
@@ -4493,7 +4493,7 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>Verkauf Fertigarzneimittel an Vertriebsgesellschaft FR03</t>
+          <t>Sale of finished pharmaceuticals to distributor FR03</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
@@ -4538,7 +4538,7 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>Verkauf Fertigarzneimittel an Vertriebsgesellschaft FR03</t>
+          <t>Sale of finished pharmaceuticals to distributor FR03</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
@@ -4583,7 +4583,7 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>Verkauf Fertigarzneimittel an Vertriebsgesellschaft FR03</t>
+          <t>Sale of finished pharmaceuticals to distributor FR03</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
@@ -4628,7 +4628,7 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>Verkauf Fertigarzneimittel an Vertriebsgesellschaft FR03</t>
+          <t>Sale of finished pharmaceuticals to distributor FR03</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
@@ -4673,7 +4673,7 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>Verkauf Fertigarzneimittel an Vertriebsgesellschaft FR03</t>
+          <t>Sale of finished pharmaceuticals to distributor FR03</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
@@ -4718,7 +4718,7 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>Verkauf Fertigarzneimittel an Vertriebsgesellschaft FR03</t>
+          <t>Sale of finished pharmaceuticals to distributor FR03</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
@@ -4763,7 +4763,7 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>Verkauf Fertigarzneimittel an Vertriebsgesellschaft FR03</t>
+          <t>Sale of finished pharmaceuticals to distributor FR03</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
@@ -4808,7 +4808,7 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>Verkauf Fertigware an Grosshaendler OCP Pharma France</t>
+          <t>Sale of finished goods to wholesaler OCP Pharma France</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
@@ -4849,7 +4849,7 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>Verkauf Fertigware an Grosshaendler Pharmacie Centrale Lyon</t>
+          <t>Sale of finished goods to wholesaler Pharmacie Centrale Lyon</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
@@ -4890,7 +4890,7 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>Verkauf Fertigware an Grosshaendler CERP Rouen Distribution</t>
+          <t>Sale of finished goods to wholesaler CERP Rouen Distribution</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
@@ -4931,7 +4931,7 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>Verkauf Fertigware an Grosshaendler CERP Rouen Distribution</t>
+          <t>Sale of finished goods to wholesaler CERP Rouen Distribution</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
@@ -4972,7 +4972,7 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>Verkauf Fertigware an Grosshaendler OCP Pharma France</t>
+          <t>Sale of finished goods to wholesaler OCP Pharma France</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
@@ -5013,7 +5013,7 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>Verkauf Fertigware an Grosshaendler CERP Rouen Distribution</t>
+          <t>Sale of finished goods to wholesaler CERP Rouen Distribution</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
@@ -5054,7 +5054,7 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>Verkauf Fertigware an Grosshaendler CERP Rouen Distribution</t>
+          <t>Sale of finished goods to wholesaler CERP Rouen Distribution</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
@@ -5095,7 +5095,7 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>Verkauf Fertigware an Grosshaendler CERP Rouen Distribution</t>
+          <t>Sale of finished goods to wholesaler CERP Rouen Distribution</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
@@ -5136,7 +5136,7 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>Verkauf Fertigware an Grosshaendler CERP Rouen Distribution</t>
+          <t>Sale of finished goods to wholesaler CERP Rouen Distribution</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
@@ -5177,7 +5177,7 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>Verkauf Fertigware an Grosshaendler CERP Rouen Distribution</t>
+          <t>Sale of finished goods to wholesaler CERP Rouen Distribution</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
@@ -5218,7 +5218,7 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>Verkauf Fertigware an Grosshaendler Pharmacie Centrale Lyon</t>
+          <t>Sale of finished goods to wholesaler Pharmacie Centrale Lyon</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
@@ -5259,7 +5259,7 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>Verkauf Fertigware an Grosshaendler Pharmacie Centrale Lyon</t>
+          <t>Sale of finished goods to wholesaler Pharmacie Centrale Lyon</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
@@ -5300,7 +5300,7 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>Verkauf Fertigware an Grosshaendler CERP Rouen Distribution</t>
+          <t>Sale of finished goods to wholesaler CERP Rouen Distribution</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
@@ -5341,7 +5341,7 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>Verkauf Fertigware an Grosshaendler CERP Rouen Distribution</t>
+          <t>Sale of finished goods to wholesaler CERP Rouen Distribution</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
@@ -5382,7 +5382,7 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>Verkauf Fertigware an Grosshaendler OCP Pharma France</t>
+          <t>Sale of finished goods to wholesaler OCP Pharma France</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
@@ -5423,7 +5423,7 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>Verkauf Fertigware an Grosshaendler CERP Rouen Distribution</t>
+          <t>Sale of finished goods to wholesaler CERP Rouen Distribution</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
@@ -5464,7 +5464,7 @@
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>Verkauf Fertigware an Grosshaendler OCP Pharma France</t>
+          <t>Sale of finished goods to wholesaler OCP Pharma France</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
@@ -5505,7 +5505,7 @@
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>Verkauf Fertigware an Grosshaendler Pharmacie Centrale Lyon</t>
+          <t>Sale of finished goods to wholesaler Pharmacie Centrale Lyon</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
@@ -5546,7 +5546,7 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>Verkauf Fertigware an Grosshaendler CERP Rouen Distribution</t>
+          <t>Sale of finished goods to wholesaler CERP Rouen Distribution</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
@@ -5587,7 +5587,7 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>Verkauf Fertigware an Grosshaendler OCP Pharma France</t>
+          <t>Sale of finished goods to wholesaler OCP Pharma France</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
@@ -5628,7 +5628,7 @@
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>Verkauf Fertigware an Grosshaendler Pharmacie Centrale Lyon</t>
+          <t>Sale of finished goods to wholesaler Pharmacie Centrale Lyon</t>
         </is>
       </c>
       <c r="D122" t="inlineStr">
@@ -5669,7 +5669,7 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>Verkauf Fertigware an Grosshaendler Pharmacie Centrale Lyon</t>
+          <t>Sale of finished goods to wholesaler Pharmacie Centrale Lyon</t>
         </is>
       </c>
       <c r="D123" t="inlineStr">
@@ -5710,7 +5710,7 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>Verkauf Fertigware an Grosshaendler Pharmacie Centrale Lyon</t>
+          <t>Sale of finished goods to wholesaler Pharmacie Centrale Lyon</t>
         </is>
       </c>
       <c r="D124" t="inlineStr">
@@ -5751,7 +5751,7 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>Verkauf Fertigware an Grosshaendler OCP Pharma France</t>
+          <t>Sale of finished goods to wholesaler OCP Pharma France</t>
         </is>
       </c>
       <c r="D125" t="inlineStr">
@@ -5792,7 +5792,7 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>Verkauf Fertigware an Grosshaendler CERP Rouen Distribution</t>
+          <t>Sale of finished goods to wholesaler CERP Rouen Distribution</t>
         </is>
       </c>
       <c r="D126" t="inlineStr">
@@ -5833,7 +5833,7 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>Verkauf Fertigware an Grosshaendler OCP Pharma France</t>
+          <t>Sale of finished goods to wholesaler OCP Pharma France</t>
         </is>
       </c>
       <c r="D127" t="inlineStr">
@@ -5874,7 +5874,7 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>Gutschrift Retoure Grosshandel</t>
+          <t>Credit note wholesale return</t>
         </is>
       </c>
       <c r="D128" t="inlineStr">
@@ -5915,7 +5915,7 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>Verkauf Fertigarzneimittel an Vertriebsgesellschaft SG01</t>
+          <t>Sale of finished pharmaceuticals to distributor SG01</t>
         </is>
       </c>
       <c r="D129" t="inlineStr">
@@ -5960,7 +5960,7 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>Verkauf Fertigarzneimittel an Vertriebsgesellschaft SG01</t>
+          <t>Sale of finished pharmaceuticals to distributor SG01</t>
         </is>
       </c>
       <c r="D130" t="inlineStr">
@@ -6005,7 +6005,7 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>Verkauf Fertigarzneimittel an Vertriebsgesellschaft SG01</t>
+          <t>Sale of finished pharmaceuticals to distributor SG01</t>
         </is>
       </c>
       <c r="D131" t="inlineStr">
@@ -6050,7 +6050,7 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>Verkauf Fertigarzneimittel an Vertriebsgesellschaft SG01</t>
+          <t>Sale of finished pharmaceuticals to distributor SG01</t>
         </is>
       </c>
       <c r="D132" t="inlineStr">
@@ -6095,7 +6095,7 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>Verkauf Fertigarzneimittel an Vertriebsgesellschaft SG01</t>
+          <t>Sale of finished pharmaceuticals to distributor SG01</t>
         </is>
       </c>
       <c r="D133" t="inlineStr">
@@ -6140,7 +6140,7 @@
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>Verkauf Fertigarzneimittel an Vertriebsgesellschaft SG01</t>
+          <t>Sale of finished pharmaceuticals to distributor SG01</t>
         </is>
       </c>
       <c r="D134" t="inlineStr">
@@ -6185,7 +6185,7 @@
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>Verkauf Fertigarzneimittel an Vertriebsgesellschaft SG01</t>
+          <t>Sale of finished pharmaceuticals to distributor SG01</t>
         </is>
       </c>
       <c r="D135" t="inlineStr">
@@ -6230,7 +6230,7 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>Verkauf Fertigarzneimittel an Vertriebsgesellschaft SG01</t>
+          <t>Sale of finished pharmaceuticals to distributor SG01</t>
         </is>
       </c>
       <c r="D136" t="inlineStr">
@@ -6275,7 +6275,7 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>Verkauf Fertigarzneimittel an Vertriebsgesellschaft SG01</t>
+          <t>Sale of finished pharmaceuticals to distributor SG01</t>
         </is>
       </c>
       <c r="D137" t="inlineStr">
@@ -6320,7 +6320,7 @@
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>Verkauf Fertigarzneimittel an Vertriebsgesellschaft SG01</t>
+          <t>Sale of finished pharmaceuticals to distributor SG01</t>
         </is>
       </c>
       <c r="D138" t="inlineStr">
@@ -6365,7 +6365,7 @@
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>Verkauf Fertigarzneimittel an Vertriebsgesellschaft SG01</t>
+          <t>Sale of finished pharmaceuticals to distributor SG01</t>
         </is>
       </c>
       <c r="D139" t="inlineStr">
@@ -6410,7 +6410,7 @@
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>Verkauf Fertigarzneimittel an Vertriebsgesellschaft SG01</t>
+          <t>Sale of finished pharmaceuticals to distributor SG01</t>
         </is>
       </c>
       <c r="D140" t="inlineStr">
@@ -6455,7 +6455,7 @@
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>Verkauf Fertigarzneimittel an Vertriebsgesellschaft SG01</t>
+          <t>Sale of finished pharmaceuticals to distributor SG01</t>
         </is>
       </c>
       <c r="D141" t="inlineStr">
@@ -6500,7 +6500,7 @@
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>Verkauf Fertigarzneimittel an Vertriebsgesellschaft SG01</t>
+          <t>Sale of finished pharmaceuticals to distributor SG01</t>
         </is>
       </c>
       <c r="D142" t="inlineStr">
@@ -6545,7 +6545,7 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>Verkauf Fertigarzneimittel an Vertriebsgesellschaft SG01</t>
+          <t>Sale of finished pharmaceuticals to distributor SG01</t>
         </is>
       </c>
       <c r="D143" t="inlineStr">
@@ -6590,7 +6590,7 @@
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>Verkauf Fertigarzneimittel an Vertriebsgesellschaft SG01</t>
+          <t>Sale of finished pharmaceuticals to distributor SG01</t>
         </is>
       </c>
       <c r="D144" t="inlineStr">
@@ -6635,7 +6635,7 @@
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>Verkauf Fertigarzneimittel an Vertriebsgesellschaft SG01</t>
+          <t>Sale of finished pharmaceuticals to distributor SG01</t>
         </is>
       </c>
       <c r="D145" t="inlineStr">
@@ -6680,7 +6680,7 @@
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>Verkauf Fertigarzneimittel an Vertriebsgesellschaft SG01</t>
+          <t>Sale of finished pharmaceuticals to distributor SG01</t>
         </is>
       </c>
       <c r="D146" t="inlineStr">
@@ -6725,7 +6725,7 @@
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>Verkauf Fertigarzneimittel an Vertriebsgesellschaft SG01</t>
+          <t>Sale of finished pharmaceuticals to distributor SG01</t>
         </is>
       </c>
       <c r="D147" t="inlineStr">
@@ -6770,7 +6770,7 @@
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>Verkauf Fertigware an Grosshaendler Singapore MedSupply</t>
+          <t>Sale of finished goods to wholesaler Singapore MedSupply</t>
         </is>
       </c>
       <c r="D148" t="inlineStr">
@@ -6811,7 +6811,7 @@
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>Verkauf Fertigware an Grosshaendler DKSH Healthcare Asia</t>
+          <t>Sale of finished goods to wholesaler DKSH Healthcare Asia</t>
         </is>
       </c>
       <c r="D149" t="inlineStr">
@@ -6852,7 +6852,7 @@
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>Verkauf Fertigware an Grosshaendler Singapore MedSupply</t>
+          <t>Sale of finished goods to wholesaler Singapore MedSupply</t>
         </is>
       </c>
       <c r="D150" t="inlineStr">
@@ -6893,7 +6893,7 @@
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>Verkauf Fertigware an Grosshaendler DKSH Healthcare Asia</t>
+          <t>Sale of finished goods to wholesaler DKSH Healthcare Asia</t>
         </is>
       </c>
       <c r="D151" t="inlineStr">
@@ -6934,7 +6934,7 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>Verkauf Fertigware an Grosshaendler DKSH Healthcare Asia</t>
+          <t>Sale of finished goods to wholesaler DKSH Healthcare Asia</t>
         </is>
       </c>
       <c r="D152" t="inlineStr">
@@ -6975,7 +6975,7 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>Verkauf Fertigware an Grosshaendler DKSH Healthcare Asia</t>
+          <t>Sale of finished goods to wholesaler DKSH Healthcare Asia</t>
         </is>
       </c>
       <c r="D153" t="inlineStr">
@@ -7016,7 +7016,7 @@
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>Verkauf Fertigware an Grosshaendler Zuellig Pharma Singapore</t>
+          <t>Sale of finished goods to wholesaler Zuellig Pharma Singapore</t>
         </is>
       </c>
       <c r="D154" t="inlineStr">
@@ -7057,7 +7057,7 @@
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>Verkauf Fertigware an Grosshaendler Zuellig Pharma Singapore</t>
+          <t>Sale of finished goods to wholesaler Zuellig Pharma Singapore</t>
         </is>
       </c>
       <c r="D155" t="inlineStr">
@@ -7098,7 +7098,7 @@
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>Verkauf Fertigware an Grosshaendler DKSH Healthcare Asia</t>
+          <t>Sale of finished goods to wholesaler DKSH Healthcare Asia</t>
         </is>
       </c>
       <c r="D156" t="inlineStr">
@@ -7139,7 +7139,7 @@
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>Verkauf Fertigware an Grosshaendler Singapore MedSupply</t>
+          <t>Sale of finished goods to wholesaler Singapore MedSupply</t>
         </is>
       </c>
       <c r="D157" t="inlineStr">
@@ -7180,7 +7180,7 @@
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>Verkauf Fertigware an Grosshaendler Singapore MedSupply</t>
+          <t>Sale of finished goods to wholesaler Singapore MedSupply</t>
         </is>
       </c>
       <c r="D158" t="inlineStr">
@@ -7221,7 +7221,7 @@
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>Verkauf Fertigware an Grosshaendler Singapore MedSupply</t>
+          <t>Sale of finished goods to wholesaler Singapore MedSupply</t>
         </is>
       </c>
       <c r="D159" t="inlineStr">
@@ -7262,7 +7262,7 @@
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>Verkauf Fertigware an Grosshaendler Zuellig Pharma Singapore</t>
+          <t>Sale of finished goods to wholesaler Zuellig Pharma Singapore</t>
         </is>
       </c>
       <c r="D160" t="inlineStr">
@@ -7303,7 +7303,7 @@
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>Verkauf Fertigware an Grosshaendler Zuellig Pharma Singapore</t>
+          <t>Sale of finished goods to wholesaler Zuellig Pharma Singapore</t>
         </is>
       </c>
       <c r="D161" t="inlineStr">
@@ -7344,7 +7344,7 @@
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>Verkauf Fertigware an Grosshaendler Zuellig Pharma Singapore</t>
+          <t>Sale of finished goods to wholesaler Zuellig Pharma Singapore</t>
         </is>
       </c>
       <c r="D162" t="inlineStr">
@@ -7385,7 +7385,7 @@
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>Verkauf Fertigware an Grosshaendler Singapore MedSupply</t>
+          <t>Sale of finished goods to wholesaler Singapore MedSupply</t>
         </is>
       </c>
       <c r="D163" t="inlineStr">
@@ -7426,7 +7426,7 @@
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>Verkauf Fertigware an Grosshaendler DKSH Healthcare Asia</t>
+          <t>Sale of finished goods to wholesaler DKSH Healthcare Asia</t>
         </is>
       </c>
       <c r="D164" t="inlineStr">
@@ -7467,7 +7467,7 @@
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>Verkauf Fertigware an Grosshaendler DKSH Healthcare Asia</t>
+          <t>Sale of finished goods to wholesaler DKSH Healthcare Asia</t>
         </is>
       </c>
       <c r="D165" t="inlineStr">
@@ -7508,7 +7508,7 @@
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>Verkauf Fertigware an Grosshaendler DKSH Healthcare Asia</t>
+          <t>Sale of finished goods to wholesaler DKSH Healthcare Asia</t>
         </is>
       </c>
       <c r="D166" t="inlineStr">
@@ -7549,7 +7549,7 @@
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>Verkauf Fertigware an Grosshaendler Zuellig Pharma Singapore</t>
+          <t>Sale of finished goods to wholesaler Zuellig Pharma Singapore</t>
         </is>
       </c>
       <c r="D167" t="inlineStr">
@@ -7590,7 +7590,7 @@
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>Verkauf Fertigware an Grosshaendler DKSH Healthcare Asia</t>
+          <t>Sale of finished goods to wholesaler DKSH Healthcare Asia</t>
         </is>
       </c>
       <c r="D168" t="inlineStr">
@@ -7631,7 +7631,7 @@
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>Verkauf Fertigware an Grosshaendler Singapore MedSupply</t>
+          <t>Sale of finished goods to wholesaler Singapore MedSupply</t>
         </is>
       </c>
       <c r="D169" t="inlineStr">
@@ -7672,7 +7672,7 @@
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>Gutschrift Retoure Grosshandel</t>
+          <t>Credit note wholesale return</t>
         </is>
       </c>
       <c r="D170" t="inlineStr">
@@ -7713,7 +7713,7 @@
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>Lohnfertigungsgebuehr API-Produktion</t>
+          <t>Contract manufacturing fee API production</t>
         </is>
       </c>
       <c r="D171" t="inlineStr">
@@ -7758,7 +7758,7 @@
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>Lohnfertigungsgebuehr API-Produktion</t>
+          <t>Contract manufacturing fee API production</t>
         </is>
       </c>
       <c r="D172" t="inlineStr">
@@ -7803,7 +7803,7 @@
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>Lohnfertigungsgebuehr API-Produktion</t>
+          <t>Contract manufacturing fee API production</t>
         </is>
       </c>
       <c r="D173" t="inlineStr">
@@ -7848,7 +7848,7 @@
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>Lohnfertigungsgebuehr API-Produktion</t>
+          <t>Contract manufacturing fee API production</t>
         </is>
       </c>
       <c r="D174" t="inlineStr">
@@ -7893,7 +7893,7 @@
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>Lohnfertigungsgebuehr API-Produktion</t>
+          <t>Contract manufacturing fee API production</t>
         </is>
       </c>
       <c r="D175" t="inlineStr">
@@ -7938,7 +7938,7 @@
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>Lohnfertigungsgebuehr API-Produktion</t>
+          <t>Contract manufacturing fee API production</t>
         </is>
       </c>
       <c r="D176" t="inlineStr">
@@ -7983,7 +7983,7 @@
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>Lohnfertigungsgebuehr API-Produktion</t>
+          <t>Contract manufacturing fee API production</t>
         </is>
       </c>
       <c r="D177" t="inlineStr">
@@ -8028,7 +8028,7 @@
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>Lohnfertigungsgebuehr API-Produktion</t>
+          <t>Contract manufacturing fee API production</t>
         </is>
       </c>
       <c r="D178" t="inlineStr">
@@ -8073,7 +8073,7 @@
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>Lohnfertigungsgebuehr API-Produktion</t>
+          <t>Contract manufacturing fee API production</t>
         </is>
       </c>
       <c r="D179" t="inlineStr">
@@ -8118,7 +8118,7 @@
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>Lohnfertigungsgebuehr API-Produktion</t>
+          <t>Contract manufacturing fee API production</t>
         </is>
       </c>
       <c r="D180" t="inlineStr">
@@ -8163,7 +8163,7 @@
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>Lohnfertigungsgebuehr API-Produktion</t>
+          <t>Contract manufacturing fee API production</t>
         </is>
       </c>
       <c r="D181" t="inlineStr">
@@ -8208,7 +8208,7 @@
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>Lohnfertigungsgebuehr API-Produktion</t>
+          <t>Contract manufacturing fee API production</t>
         </is>
       </c>
       <c r="D182" t="inlineStr">
@@ -8253,7 +8253,7 @@
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>Sonstige Kosten - noch nicht klassifiziert</t>
+          <t>Other costs - not classified</t>
         </is>
       </c>
       <c r="D183" t="inlineStr">
@@ -8294,7 +8294,7 @@
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>Sonstige Kosten - noch nicht klassifiziert</t>
+          <t>Other costs - not classified</t>
         </is>
       </c>
       <c r="D184" t="inlineStr">
@@ -8335,7 +8335,7 @@
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>Sonstige Kosten - noch nicht klassifiziert</t>
+          <t>Other costs - not classified</t>
         </is>
       </c>
       <c r="D185" t="inlineStr">
@@ -8380,7 +8380,7 @@
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>Sonstige Kosten - noch nicht klassifiziert</t>
+          <t>Other costs - not classified</t>
         </is>
       </c>
       <c r="D186" t="inlineStr">
@@ -8421,7 +8421,7 @@
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>Sonstige Kosten - noch nicht klassifiziert</t>
+          <t>Other costs - not classified</t>
         </is>
       </c>
       <c r="D187" t="inlineStr">
@@ -8466,7 +8466,7 @@
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>Sonstige Kosten - noch nicht klassifiziert</t>
+          <t>Other costs - not classified</t>
         </is>
       </c>
       <c r="D188" t="inlineStr">
@@ -8511,7 +8511,7 @@
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>Sonstige Kosten - noch nicht klassifiziert</t>
+          <t>Other costs - not classified</t>
         </is>
       </c>
       <c r="D189" t="inlineStr">
@@ -8556,7 +8556,7 @@
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t>Sonstige Kosten - noch nicht klassifiziert</t>
+          <t>Other costs - not classified</t>
         </is>
       </c>
       <c r="D190" t="inlineStr">
@@ -8601,7 +8601,7 @@
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>Sonstige Kosten - noch nicht klassifiziert</t>
+          <t>Other costs - not classified</t>
         </is>
       </c>
       <c r="D191" t="inlineStr">
@@ -8642,7 +8642,7 @@
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>Sonstige Kosten - noch nicht klassifiziert</t>
+          <t>Other costs - not classified</t>
         </is>
       </c>
       <c r="D192" t="inlineStr">
@@ -8687,7 +8687,7 @@
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>Sonstige Kosten - noch nicht klassifiziert</t>
+          <t>Other costs - not classified</t>
         </is>
       </c>
       <c r="D193" t="inlineStr">
@@ -8732,7 +8732,7 @@
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>Sonstige Kosten - noch nicht klassifiziert</t>
+          <t>Other costs - not classified</t>
         </is>
       </c>
       <c r="D194" t="inlineStr">
@@ -8777,7 +8777,7 @@
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>Sonstige Kosten - noch nicht klassifiziert</t>
+          <t>Other costs - not classified</t>
         </is>
       </c>
       <c r="D195" t="inlineStr">
@@ -8822,7 +8822,7 @@
       </c>
       <c r="C196" t="inlineStr">
         <is>
-          <t>Sonstige Kosten - noch nicht klassifiziert</t>
+          <t>Other costs - not classified</t>
         </is>
       </c>
       <c r="D196" t="inlineStr">
@@ -8867,7 +8867,7 @@
       </c>
       <c r="C197" t="inlineStr">
         <is>
-          <t>Sonstige Kosten - noch nicht klassifiziert</t>
+          <t>Other costs - not classified</t>
         </is>
       </c>
       <c r="D197" t="inlineStr">
@@ -8908,7 +8908,7 @@
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>Sonstige Kosten - noch nicht klassifiziert</t>
+          <t>Other costs - not classified</t>
         </is>
       </c>
       <c r="D198" t="inlineStr">
@@ -8953,7 +8953,7 @@
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t>Sonstige Kosten - noch nicht klassifiziert</t>
+          <t>Other costs - not classified</t>
         </is>
       </c>
       <c r="D199" t="inlineStr">
@@ -8998,7 +8998,7 @@
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>Sonstige Kosten - noch nicht klassifiziert</t>
+          <t>Other costs - not classified</t>
         </is>
       </c>
       <c r="D200" t="inlineStr">
@@ -9043,7 +9043,7 @@
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>Sonstige Kosten - noch nicht klassifiziert</t>
+          <t>Other costs - not classified</t>
         </is>
       </c>
       <c r="D201" t="inlineStr">
@@ -9088,7 +9088,7 @@
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>Sonstige Kosten - noch nicht klassifiziert</t>
+          <t>Other costs - not classified</t>
         </is>
       </c>
       <c r="D202" t="inlineStr">
@@ -9133,7 +9133,7 @@
       </c>
       <c r="C203" t="inlineStr">
         <is>
-          <t>Sonstige Kosten - noch nicht klassifiziert</t>
+          <t>Other costs - not classified</t>
         </is>
       </c>
       <c r="D203" t="inlineStr">
@@ -9174,7 +9174,7 @@
       </c>
       <c r="C204" t="inlineStr">
         <is>
-          <t>Sonstige Kosten - noch nicht klassifiziert</t>
+          <t>Other costs - not classified</t>
         </is>
       </c>
       <c r="D204" t="inlineStr">
@@ -9219,7 +9219,7 @@
       </c>
       <c r="C205" t="inlineStr">
         <is>
-          <t>Sonstige Kosten - noch nicht klassifiziert</t>
+          <t>Other costs - not classified</t>
         </is>
       </c>
       <c r="D205" t="inlineStr">
@@ -9264,7 +9264,7 @@
       </c>
       <c r="C206" t="inlineStr">
         <is>
-          <t>Sonstige Kosten - noch nicht klassifiziert</t>
+          <t>Other costs - not classified</t>
         </is>
       </c>
       <c r="D206" t="inlineStr">
@@ -9309,7 +9309,7 @@
       </c>
       <c r="C207" t="inlineStr">
         <is>
-          <t>Sonstige Kosten - noch nicht klassifiziert</t>
+          <t>Other costs - not classified</t>
         </is>
       </c>
       <c r="D207" t="inlineStr">
@@ -9354,7 +9354,7 @@
       </c>
       <c r="C208" t="inlineStr">
         <is>
-          <t>Sonstige Kosten - noch nicht klassifiziert</t>
+          <t>Other costs - not classified</t>
         </is>
       </c>
       <c r="D208" t="inlineStr">
@@ -9399,7 +9399,7 @@
       </c>
       <c r="C209" t="inlineStr">
         <is>
-          <t>Sonstige Kosten - noch nicht klassifiziert</t>
+          <t>Other costs - not classified</t>
         </is>
       </c>
       <c r="D209" t="inlineStr">
@@ -9444,7 +9444,7 @@
       </c>
       <c r="C210" t="inlineStr">
         <is>
-          <t>Sonstige Kosten - noch nicht klassifiziert</t>
+          <t>Other costs - not classified</t>
         </is>
       </c>
       <c r="D210" t="inlineStr">
@@ -9489,7 +9489,7 @@
       </c>
       <c r="C211" t="inlineStr">
         <is>
-          <t>Sonstige Kosten - noch nicht klassifiziert</t>
+          <t>Other costs - not classified</t>
         </is>
       </c>
       <c r="D211" t="inlineStr">
@@ -9534,7 +9534,7 @@
       </c>
       <c r="C212" t="inlineStr">
         <is>
-          <t>Sonstige Kosten - noch nicht klassifiziert</t>
+          <t>Other costs - not classified</t>
         </is>
       </c>
       <c r="D212" t="inlineStr">
@@ -9575,7 +9575,7 @@
       </c>
       <c r="C213" t="inlineStr">
         <is>
-          <t>Sonstige Kosten - noch nicht klassifiziert</t>
+          <t>Other costs - not classified</t>
         </is>
       </c>
       <c r="D213" t="inlineStr">
@@ -9620,7 +9620,7 @@
       </c>
       <c r="C214" t="inlineStr">
         <is>
-          <t>Sonstige Kosten - noch nicht klassifiziert</t>
+          <t>Other costs - not classified</t>
         </is>
       </c>
       <c r="D214" t="inlineStr">

</xml_diff>